<commit_message>
Aplicación de refactorización FASES 1 y 2
</commit_message>
<xml_diff>
--- a/Sistema de Teleprompter/Excel/prompter_intro.xlsx
+++ b/Sistema de Teleprompter/Excel/prompter_intro.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\STP\Sistema de Teleprompter\Excel\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CB4996A-FE9A-49F3-A557-40B04C2CF347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="72" windowWidth="22116" windowHeight="10080"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -16,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>NUMERO_GUION</t>
   </si>
@@ -34,12 +40,18 @@
   </si>
   <si>
     <t>BIENEVENIDOS A ESTE NUEVO PROYECTO DE TELECOMUNICACIONES</t>
+  </si>
+  <si>
+    <t>DURACION</t>
+  </si>
+  <si>
+    <t>NOTAS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -167,13 +179,13 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -186,14 +198,17 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -231,7 +246,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -303,7 +318,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -476,16 +491,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C21"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.77734375" customWidth="1"/>
     <col min="2" max="2" width="33.33203125" customWidth="1"/>
     <col min="3" max="3" width="45.5546875" customWidth="1"/>
+    <col min="4" max="4" width="43.6640625" customWidth="1"/>
+    <col min="5" max="5" width="35.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -495,89 +512,95 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="123.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" ht="123.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C3" s="5"/>
     </row>
-    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="6"/>
-    </row>
-    <row r="5" spans="1:3" ht="122.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C4" s="4"/>
+    </row>
+    <row r="5" spans="1:5" ht="122.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C5" s="5"/>
     </row>
-    <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>3</v>
       </c>
       <c r="B6" s="1"/>
-      <c r="C6" s="6"/>
-    </row>
-    <row r="7" spans="1:3" ht="126.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C6" s="4"/>
+    </row>
+    <row r="7" spans="1:5" ht="126.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C7" s="5"/>
     </row>
-    <row r="8" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>4</v>
       </c>
       <c r="B8" s="1"/>
-      <c r="C8" s="6"/>
-    </row>
-    <row r="9" spans="1:3" ht="152.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C8" s="4"/>
+    </row>
+    <row r="9" spans="1:5" ht="152.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C9" s="5"/>
     </row>
-    <row r="10" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>5</v>
       </c>
       <c r="B10" s="1"/>
-      <c r="C10" s="6"/>
-    </row>
-    <row r="11" spans="1:3" ht="128.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C10" s="4"/>
+    </row>
+    <row r="11" spans="1:5" ht="128.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C11" s="5"/>
     </row>
-    <row r="12" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>6</v>
       </c>
       <c r="B12" s="1"/>
-      <c r="C12" s="6"/>
-    </row>
-    <row r="13" spans="1:3" ht="183" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C12" s="4"/>
+    </row>
+    <row r="13" spans="1:5" ht="183" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C13" s="5"/>
     </row>
-    <row r="14" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>7</v>
       </c>
       <c r="B14" s="1"/>
-      <c r="C14" s="6"/>
-    </row>
-    <row r="15" spans="1:3" ht="111" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C14" s="4"/>
+    </row>
+    <row r="15" spans="1:5" ht="111" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C15" s="5"/>
     </row>
-    <row r="16" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>8</v>
       </c>
       <c r="B16" s="1"/>
-      <c r="C16" s="6"/>
+      <c r="C16" s="4"/>
     </row>
     <row r="17" spans="1:3" ht="117.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C17" s="5"/>
@@ -587,7 +610,7 @@
         <v>9</v>
       </c>
       <c r="B18" s="1"/>
-      <c r="C18" s="6"/>
+      <c r="C18" s="4"/>
     </row>
     <row r="19" spans="1:3" ht="141.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C19" s="5"/>
@@ -597,7 +620,7 @@
         <v>10</v>
       </c>
       <c r="B20" s="1"/>
-      <c r="C20" s="6"/>
+      <c r="C20" s="4"/>
     </row>
     <row r="21" spans="1:3" ht="147" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C21" s="5"/>
@@ -621,7 +644,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
@@ -630,7 +653,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>

</xml_diff>